<commit_message>
Configurar integração Duolingo de Admin
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -22145,9 +22145,13 @@
           <t>{}</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>DarleiD</t>
+        </is>
+      </c>
       <c r="L2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M2" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Atalho 1 clique: English Live concluído (Admin)
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -517,13 +517,21 @@
         <v>30</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="J2" t="b">
-        <v>0</v>
-      </c>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Marcado via atalho de 1 clique (English Live)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-09-29 20:12</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">

</xml_diff>